<commit_message>
Fix bug + update data source
</commit_message>
<xml_diff>
--- a/docs/release-todo.xlsx
+++ b/docs/release-todo.xlsx
@@ -1915,11 +1915,15 @@
       </c>
       <c r="J5" s="20" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Đang làm</t>
         </is>
       </c>
       <c r="K5" s="21" t="inlineStr"/>
-      <c r="L5" s="21" t="inlineStr"/>
+      <c r="L5" s="21" t="inlineStr">
+        <is>
+          <t>Code xong 18/10/2026: tối đa 3 lượt đổi/ngày (reroll + adopt dùng chung), skippedCount +1 tối đa 1 lần/ngày, PersistedState v2 (swapsUsed). Review APPROVE. Còn QA tay: xem docs/plans/T-04_T-35.md (Test report).</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="17" t="inlineStr">
@@ -1967,11 +1971,15 @@
       </c>
       <c r="J6" s="20" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Đang làm</t>
         </is>
       </c>
       <c r="K6" s="21" t="inlineStr"/>
-      <c r="L6" s="21" t="inlineStr"/>
+      <c r="L6" s="21" t="inlineStr">
+        <is>
+          <t>Code xong 19/10/2026: favorites lưu bền (PersistedState v3, favoriteQuoteIds), chip "Tất cả / Đã thích" ở S14, "Xóa tất cả dữ liệu" xoá luôn favorites. Review APPROVE. Còn QA tay: xem docs/plans/T-05.md.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="17" t="inlineStr">
@@ -2019,11 +2027,15 @@
       </c>
       <c r="J7" s="20" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Đang làm</t>
         </is>
       </c>
       <c r="K7" s="21" t="inlineStr"/>
-      <c r="L7" s="21" t="inlineStr"/>
+      <c r="L7" s="21" t="inlineStr">
+        <is>
+          <t>Code xong 19/10/2026 (chốt: rung + âm hệ thống, không tệp âm thanh): rung khi hoàn thành / lên level (mạnh hơn) / chọn lĩnh vực, âm hệ thống ngắn khi nhận thưởng, preview khi bật toggle; toggle cũng tắt âm thông báo Android. Không thêm quyền. Review APPROVE. Còn QA tay trên máy thật: xem docs/plans/T-06.md.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="17" t="inlineStr">
@@ -2071,11 +2083,15 @@
       </c>
       <c r="J8" s="20" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Đang làm</t>
         </is>
       </c>
       <c r="K8" s="21" t="inlineStr"/>
-      <c r="L8" s="21" t="inlineStr"/>
+      <c r="L8" s="21" t="inlineStr">
+        <is>
+          <t>Code xong 19/10/2026: system bar theo theme trong app (đổi ngay cả khi đổi dark mode hệ thống), thẻ chia sẻ luôn tối trên cả hai nền tảng (sửa chữ khó đọc ở theme Sáng). Review APPROVE sau 1 vòng sửa. Còn QA tay: xem docs/plans/T-07_T-29.md.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="17" t="inlineStr">
@@ -2123,11 +2139,15 @@
       </c>
       <c r="J9" s="20" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Đang làm</t>
         </is>
       </c>
       <c r="K9" s="21" t="inlineStr"/>
-      <c r="L9" s="21" t="inlineStr"/>
+      <c r="L9" s="21" t="inlineStr">
+        <is>
+          <t>Code xong 18/10/2026: ReminderPlanner (shared) — đã xong hôm nay thì không nhắc, gỡ thông báo đã hiện khi hoàn thành, copy "giữ chuỗi" khi chuỗi tới hôm qua ≥ 3. Review APPROVE. Còn QA tay: xem docs/plans/T-08_T-09.md.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="17" t="inlineStr">
@@ -2175,11 +2195,15 @@
       </c>
       <c r="J10" s="20" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Đang làm</t>
         </is>
       </c>
       <c r="K10" s="21" t="inlineStr"/>
-      <c r="L10" s="21" t="inlineStr"/>
+      <c r="L10" s="21" t="inlineStr">
+        <is>
+          <t>Code xong 18/10/2026: Android BootReceiver nhận TIME_SET/TIMEZONE_CHANGED; iOS dayIndex theo ngày địa phương, dựng lại lịch khi sang ngày/hoàn thành, nhắc cuối cửa sổ 14 ngày "Lâu rồi không gặp". Không dùng LOCKED_BOOT_COMPLETED. Review APPROVE. Còn QA tay (Android #5–6 khi app bị kill): xem docs/plans/T-08_T-09.md.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="17" t="inlineStr">
@@ -2331,11 +2355,15 @@
       </c>
       <c r="J13" s="20" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Đang làm</t>
         </is>
       </c>
       <c r="K13" s="21" t="inlineStr"/>
-      <c r="L13" s="21" t="inlineStr"/>
+      <c r="L13" s="21" t="inlineStr">
+        <is>
+          <t>Một phần 19/10/2026: version trong settingsFooter/aboutBody lấy từ build (BuildConfig.VERSION_NAME / CFBundleShortVersionString). Còn row Chính sách quyền riêng tư / Liên hệ / Đánh giá — chờ URL, email, link store (T-10/T-11).</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="17" t="inlineStr">
@@ -2383,11 +2411,15 @@
       </c>
       <c r="J14" s="20" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Đang làm</t>
         </is>
       </c>
       <c r="K14" s="21" t="inlineStr"/>
-      <c r="L14" s="21" t="inlineStr"/>
+      <c r="L14" s="21" t="inlineStr">
+        <is>
+          <t>Code xong 19/10/2026: "Nhập dữ liệu" ở Settings (OpenDocument / fileImporter, giới hạn 5 MB, xác nhận ghi đè kèm tóm tắt, thay toàn bộ dữ liệu), data_extraction_rules + backup_rules (oddly.xml, reminder.xml), privacy policy/store listing cập nhật. Review APPROVE sau 1 vòng sửa. Còn QA tay (bmgr, R8, alert iOS): xem docs/plans/T-13.md.</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="17" t="inlineStr">
@@ -2639,11 +2671,15 @@
       </c>
       <c r="J19" s="20" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Đang làm</t>
         </is>
       </c>
       <c r="K19" s="21" t="inlineStr"/>
-      <c r="L19" s="21" t="inlineStr"/>
+      <c r="L19" s="21" t="inlineStr">
+        <is>
+          <t>Code xong 19/10/2026: IPHONEOS_DEPLOYMENT_TARGET 18.2 → 17.0, không dùng API iOS 18. Review APPROVE. Còn QA tay trên máy/simulator iOS 17 (SwipeBack, fileImporter, ShareLink): xem docs/plans/T-28_T-18_T-22.md.</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="17" t="inlineStr">
@@ -2843,11 +2879,15 @@
       </c>
       <c r="J23" s="20" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Xong</t>
         </is>
       </c>
       <c r="K23" s="21" t="inlineStr"/>
-      <c r="L23" s="21" t="inlineStr"/>
+      <c r="L23" s="21" t="inlineStr">
+        <is>
+          <t>Xong 19/10/2026 (phương án tối thiểu): không thêm SDK, giám sát qua Android Vitals + Xcode Organizer/TestFlight, ghi trong docs/release-process.md; privacy policy thêm câu về báo cáo chẩn đoán của hệ điều hành. Data safety/App Privacy không đổi.</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="17" t="inlineStr">
@@ -3051,11 +3091,15 @@
       </c>
       <c r="J27" s="20" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Đang làm</t>
         </is>
       </c>
       <c r="K27" s="21" t="inlineStr"/>
-      <c r="L27" s="21" t="inlineStr"/>
+      <c r="L27" s="21" t="inlineStr">
+        <is>
+          <t>Đợt A xong code 19/10/2026: quote 12 → 60 (giữ 12 id cũ, thay nội dung 6 câu còn bản quyền / gán sai tác giả), test bảo vệ id đã phát hành (PublishedContent.kt). Review APPROVE sau 1 vòng sửa. Cần duyệt docs/content-review.md + QA tay. Đợt B (thử thách 120 → 216) chưa làm. Xem docs/plans/T-26A.md.</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="17" t="inlineStr">
@@ -3107,7 +3151,11 @@
         </is>
       </c>
       <c r="K28" s="21" t="inlineStr"/>
-      <c r="L28" s="21" t="inlineStr"/>
+      <c r="L28" s="21" t="inlineStr">
+        <is>
+          <t>Danh sách quote CẦN XÁC MINH nguồn + backlog nằm ở docs/content-review.md (mục Backlog T-27), lập trong đợt T-26A 19/10/2026.</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="17" t="inlineStr">
@@ -3155,11 +3203,15 @@
       </c>
       <c r="J29" s="20" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Xong</t>
         </is>
       </c>
       <c r="K29" s="21" t="inlineStr"/>
-      <c r="L29" s="21" t="inlineStr"/>
+      <c r="L29" s="21" t="inlineStr">
+        <is>
+          <t>Xong 19/10/2026: nguồn version duy nhất iosApp/Configuration/Version.xcconfig (Gradle + Xcode cùng đọc), script tools/bump-version.sh, Android/iOS dùng chung build number, release notes song ngữ ở store-listing.md mục 6. Review APPROVE. Xem docs/plans/T-28_T-18_T-22.md.</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="17" t="inlineStr">
@@ -3207,11 +3259,15 @@
       </c>
       <c r="J30" s="20" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Đang làm</t>
         </is>
       </c>
       <c r="K30" s="21" t="inlineStr"/>
-      <c r="L30" s="21" t="inlineStr"/>
+      <c r="L30" s="21" t="inlineStr">
+        <is>
+          <t>Code xong 19/10/2026: Android dùng core-splashscreen 1.2.0, bỏ màn splash Compose (Android mất tagline, iOS giữ). Review APPROVE. Còn QA tay (một splash, icon API 24–25, bản R8): xem docs/plans/T-07_T-29.md.</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="17" t="inlineStr">
@@ -3511,11 +3567,15 @@
       </c>
       <c r="J36" s="20" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Xong</t>
         </is>
       </c>
       <c r="K36" s="21" t="inlineStr"/>
-      <c r="L36" s="21" t="inlineStr"/>
+      <c r="L36" s="21" t="inlineStr">
+        <is>
+          <t>Xong 18/10/2026: fixture V1_DOCUMENT + nhánh migrate từng bước trong OddlyRepository.decode, test đọc/import version cũ. 19/10 thêm V2_DOCUMENT (sinh bằng save) khi lên v3. Review APPROVE. Xem docs/plans/T-04_T-35.md.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:L36"/>

</xml_diff>

<commit_message>
update feature, sound, test
</commit_message>
<xml_diff>
--- a/docs/release-todo.xlsx
+++ b/docs/release-todo.xlsx
@@ -2935,11 +2935,15 @@
       </c>
       <c r="J24" s="20" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Đang làm</t>
         </is>
       </c>
       <c r="K24" s="21" t="inlineStr"/>
-      <c r="L24" s="21" t="inlineStr"/>
+      <c r="L24" s="21" t="inlineStr">
+        <is>
+          <t>Code xong 24/10/2026: T-23A nhãn/vai trò/heading/live region/vùng chạm (TalkBack + VoiceOver); T-23B Dynamic Type iOS, cuộn 6 màn, giới hạn cỡ chữ, màu chữ đạt WCAG AA (PaletteSpec dùng chung). Review APPROVE. Còn: QA tay TalkBack/VoiceOver + font scale; T-23C (neon thương hiệu làm chữ trên theme Sáng) cần duyệt bảng màu. Xem docs/plans/T-23A.md, T-23B.md.</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="17" t="inlineStr">
@@ -2987,11 +2991,15 @@
       </c>
       <c r="J25" s="20" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Xong</t>
         </is>
       </c>
       <c r="K25" s="21" t="inlineStr"/>
-      <c r="L25" s="21" t="inlineStr"/>
+      <c r="L25" s="21" t="inlineStr">
+        <is>
+          <t>Xong 24/10/2026: Android 6 Compose UI test trên emulator (smoke onboarding → hoàn thành → thưởng → Journey, T-01 giờ hoàn thành, T-02 đổi ngày ×2, T-03 một hoàn thành/ngày ×2); iOS 5 XCUITest cùng kịch bản (trừ T-01). Id dùng chung UiTestTags, đồng hồ ghim Today.pinForTesting, hook chỉ DEBUG. Review APPROVE. Lệnh chạy trong .claude/CLAUDE.md. Xem docs/plans/T-24.md.</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="17" t="inlineStr">
@@ -3097,7 +3105,7 @@
       <c r="K27" s="21" t="inlineStr"/>
       <c r="L27" s="21" t="inlineStr">
         <is>
-          <t>Đợt A xong code 19/10/2026: quote 12 → 60 (giữ 12 id cũ, thay nội dung 6 câu còn bản quyền / gán sai tác giả), test bảo vệ id đã phát hành (PublishedContent.kt). Review APPROVE sau 1 vòng sửa. Cần duyệt docs/content-review.md + QA tay. Đợt B (thử thách 120 → 216) chưa làm. Xem docs/plans/T-26A.md.</t>
+          <t>Code xong 24/10/2026: quote 12 → 60 (T-26A), thử thách 120 → 216 (T-26B1 +47 Khó, T-26B2 +29 Dễ +20 Vừa; mỗi ô lĩnh vực × độ khó 12, mỗi lĩnh vực 36). Review APPROVE. Còn: duyệt docs/content-review.md + docs/content-review-challenges.md, thêm 96 id mới vào PublishedContent.kt trước khi phát hành, QA tay. Xem docs/plans/T-26A.md, T-26B1.md, T-26B2.md.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update support references, landing page, test
</commit_message>
<xml_diff>
--- a/docs/release-todo.xlsx
+++ b/docs/release-todo.xlsx
@@ -575,7 +575,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Phân tích mã nguồn tại commit 8c842bf (nhánh master), ngày 18/10/2026. Android (Compose) + iOS (SwiftUI) + sharedLogic (KMP).</t>
+          <t>Phân tích mã nguồn ban đầu tại commit 8c842bf (18/10/2026); cập nhật tiến độ tại commit 73f905a, ngày 25/10/2026. Android (Compose) + iOS (SwiftUI) + sharedLogic (KMP).</t>
         </is>
       </c>
     </row>
@@ -758,21 +758,21 @@
     <row r="15" ht="30" customHeight="1">
       <c r="A15" s="16" t="inlineStr">
         <is>
-          <t>• Kiến trúc tốt: logic dùng chung KMP, UI native, offline hoàn toàn, song ngữ, có 67 unit test, cấu hình release (R8, privacy manifest, icon, store listing) đã chuẩn bị kỹ.</t>
+          <t>• Kiến trúc tốt: logic dùng chung KMP, UI native, offline hoàn toàn, song ngữ. Có 274 unit test shared + UI test smoke (6 Android, 5 iOS), hỗ trợ TalkBack/VoiceOver, cỡ chữ lớn, màu chữ đạt WCAG AA.</t>
         </is>
       </c>
     </row>
     <row r="16" ht="30" customHeight="1">
       <c r="A16" s="16" t="inlineStr">
         <is>
-          <t>• 3 lỗi logic phải sửa trước khi phát hành: giờ hoàn thành cứng 09:41 (T-01), ngày 'hôm nay' không cập nhật qua nửa đêm (T-02), farm XP qua 'Tất cả thử thách' (T-03).</t>
+          <t>• Đã sửa 3 lỗi logic chặn phát hành (T-01 giờ hoàn thành, T-02 đổi ngày qua nửa đêm, T-03 farm XP) và hầu hết P1 code; các task đó còn chờ QA tay trên thiết bị thật.</t>
         </is>
       </c>
     </row>
     <row r="17" ht="30" customHeight="1">
       <c r="A17" s="16" t="inlineStr">
         <is>
-          <t>• Các việc chặn phát hành còn lại là thủ tục store: placeholder thương hiệu &amp; privacy policy, signing key, tài khoản &amp; form store, screenshot, QA thiết bị thật.</t>
+          <t>• Việc chặn phát hành còn lại cần người làm: thủ tục store (T-10, T-11, T-14…T-17, T-19…T-21), duyệt nội dung + xác minh nguồn quote (T-26, T-27), duyệt bảng màu neon theme Sáng (T-23C), QA tay thiết bị thật.</t>
         </is>
       </c>
     </row>
@@ -919,7 +919,7 @@
       </c>
       <c r="G2" s="18" t="inlineStr">
         <is>
-          <t>Android 12+ sẽ hiện thêm system splash trước splash tự vẽ → có thể bị 2 lớp splash (xem T-29).</t>
+          <t>Android dùng core-splashscreen (T-29): chỉ còn 1 splash hệ thống (nền + icon), bỏ tagline; iOS giữ màn splash có tagline.</t>
         </is>
       </c>
     </row>
@@ -954,7 +954,11 @@
           <t>Hoàn thành</t>
         </is>
       </c>
-      <c r="G3" s="18" t="inlineStr"/>
+      <c r="G3" s="18" t="inlineStr">
+        <is>
+          <t>"Bỏ qua" không tắt nhắc nhở (khác "Để sau" ở màn quyền) — hành vi có sẵn, chờ quyết định sản phẩm.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="17" t="inlineStr">
@@ -1022,7 +1026,7 @@
       </c>
       <c r="G5" s="18" t="inlineStr">
         <is>
-          <t>Giờ hoàn thành đang bị gán cứng 09:41 (T-01).</t>
+          <t>Giờ hoàn thành là giờ thật (T-01). Chỉ 1 hoàn thành/ngày cho thử thách hôm nay (T-03).</t>
         </is>
       </c>
     </row>
@@ -1077,7 +1081,7 @@
       </c>
       <c r="D7" s="18" t="inlineStr">
         <is>
-          <t>Đổi thử thách hôm nay, ngẫu nhiên hoặc giới hạn trong 1 lĩnh vực. Mỗi lần đổi tăng skippedCount.</t>
+          <t>Đổi thử thách hôm nay, ngẫu nhiên hoặc giới hạn trong 1 lĩnh vực. Tối đa 3 lượt đổi/ngày (đổi và "Chọn làm thử thách hôm nay" dùng chung); skippedCount +1 tối đa 1 lần/ngày.</t>
         </is>
       </c>
       <c r="E7" s="17" t="inlineStr">
@@ -1087,12 +1091,12 @@
       </c>
       <c r="F7" s="17" t="inlineStr">
         <is>
-          <t>Một phần</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
       <c r="G7" s="18" t="inlineStr">
         <is>
-          <t>Không giới hạn số lần đổi; tỷ lệ hoàn thành bị kéo xuống (T-04).</t>
+          <t>Giới hạn lượt đổi (T-04). Còn QA tay.</t>
         </is>
       </c>
     </row>
@@ -1114,7 +1118,7 @@
       </c>
       <c r="D8" s="18" t="inlineStr">
         <is>
-          <t>Duyệt toàn bộ thư viện 120 thử thách và mở chi tiết bất kỳ thử thách nào.</t>
+          <t>Duyệt toàn bộ thư viện 216 thử thách, mở chi tiết, "Chọn làm thử thách hôm nay".</t>
         </is>
       </c>
       <c r="E8" s="17" t="inlineStr">
@@ -1124,12 +1128,12 @@
       </c>
       <c r="F8" s="17" t="inlineStr">
         <is>
-          <t>Một phần</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
       <c r="G8" s="18" t="inlineStr">
         <is>
-          <t>Có thể hoàn thành nhiều thử thách/ngày để farm XP (T-03).</t>
+          <t>Hết farm XP: 1 hoàn thành/ngày (T-03). Thư viện 216 thử thách (T-26B).</t>
         </is>
       </c>
     </row>
@@ -1287,7 +1291,7 @@
       </c>
       <c r="D13" s="18" t="inlineStr">
         <is>
-          <t>12 câu trích dẫn song ngữ, 1 câu/ngày, vuốt xem các câu khác, nút yêu thích, chia sẻ.</t>
+          <t>60 câu trích dẫn song ngữ (có nguồn), 1 câu/ngày, vuốt xem các câu khác, yêu thích lưu bền, chip lọc Tất cả / Đã thích.</t>
         </is>
       </c>
       <c r="E13" s="17" t="inlineStr">
@@ -1302,7 +1306,7 @@
       </c>
       <c r="G13" s="18" t="inlineStr">
         <is>
-          <t>Yêu thích chỉ lưu trong bộ nhớ tạm, mất khi thoát màn hình (T-05). Chỉ 12 câu → lặp lại mỗi 12 ngày.</t>
+          <t>Yêu thích lưu bền (T-05, PersistedState v3). Quote 12 → 60 (T-26A). Còn: người dùng duyệt docs/content-review.md, xác minh nguồn các câu CẦN XÁC MINH (T-27).</t>
         </is>
       </c>
     </row>
@@ -1324,7 +1328,7 @@
       </c>
       <c r="D14" s="18" t="inlineStr">
         <is>
-          <t>Theme (Hệ thống/Sáng/Tối), Ngôn ngữ (vi/en), Bật/tắt nhắc nhở, Giờ nhắc (TimePicker tự do), Âm thanh &amp; rung, Xuất dữ liệu JSON, Giới thiệu, Xóa toàn bộ dữ liệu (có xác nhận). Cảnh báo khi quyền thông báo bị tắt ở hệ thống.</t>
+          <t>Theme, Ngôn ngữ, Nhắc nhở + giờ nhắc, Âm thanh &amp; rung, Xuất / Nhập dữ liệu JSON, mục Hỗ trợ &amp; pháp lý (Đánh giá, Liên hệ &amp; góp ý, Chính sách quyền riêng tư, Giới thiệu với version từ build), Xóa toàn bộ dữ liệu. Cảnh báo khi quyền thông báo bị tắt.</t>
         </is>
       </c>
       <c r="E14" s="17" t="inlineStr">
@@ -1334,12 +1338,12 @@
       </c>
       <c r="F14" s="17" t="inlineStr">
         <is>
-          <t>Một phần</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
       <c r="G14" s="18" t="inlineStr">
         <is>
-          <t>Toggle Âm thanh &amp; rung gần như không có tác dụng (T-06). Chưa có Nhập dữ liệu, Chính sách quyền riêng tư, Liên hệ, Đánh giá app.</t>
+          <t>T-06, T-12, T-13. Hàng Đánh giá trên iOS ẩn tới khi có App Store ID (T-17).</t>
         </is>
       </c>
     </row>
@@ -1371,12 +1375,12 @@
       </c>
       <c r="F15" s="17" t="inlineStr">
         <is>
-          <t>Một phần</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
       <c r="G15" s="18" t="inlineStr">
         <is>
-          <t>Brand.SHORT_LINK / HANDLE vẫn là placeholder (T-10).</t>
+          <t>Thẻ luôn tối, khoá cỡ chữ (T-07, T-23B); link lil-dua.github.io/projects/oddly (T-10) — cần đăng trang landing trước khi phát hành.</t>
         </is>
       </c>
     </row>
@@ -1398,7 +1402,7 @@
       </c>
       <c r="D16" s="18" t="inlineStr">
         <is>
-          <t>Android: AlarmManager.setWindow (±15 phút) tự re-arm mỗi ngày, BootReceiver khôi phục sau reboot/cập nhật app, kênh thông báo riêng, icon 1% đơn sắc. iOS: lên lịch trước 14 thông báo 1 lần, làm mới khi mở app. Nội dung xoay vòng theo ngày, theo ngôn ngữ.</t>
+          <t>Android: AlarmManager tự re-arm, BootReceiver khôi phục sau reboot/cập nhật/đổi giờ/đổi múi giờ. iOS: lên lịch 14 ngày theo ngày địa phương, dựng lại khi sang ngày/hoàn thành, nhắc cuối "Lâu rồi không gặp". Không nhắc khi hôm nay đã xong; copy "giữ chuỗi" khi chuỗi ≥ 3.</t>
         </is>
       </c>
       <c r="E16" s="17" t="inlineStr">
@@ -1413,7 +1417,7 @@
       </c>
       <c r="G16" s="18" t="inlineStr">
         <is>
-          <t>Vẫn nhắc dù đã làm xong hôm nay; chưa xử lý đổi múi giờ (T-08, T-09).</t>
+          <t>Đã xử lý T-08, T-09. Còn QA tay (đổi múi giờ khi app bị kill).</t>
         </is>
       </c>
     </row>
@@ -1435,7 +1439,7 @@
       </c>
       <c r="D17" s="18" t="inlineStr">
         <is>
-          <t>Một tài liệu JSON (kotlinx.serialization) trong SharedPreferences (commit) / UserDefaults, có trường version, từ chối đọc tài liệu từ version tương lai. Không có mạng, không tài khoản.</t>
+          <t>Một tài liệu JSON (kotlinx.serialization) trong SharedPreferences (commit) / UserDefaults, version 3, migrate từng bước v1→v2→v3, từ chối version tương lai. Có Nhập dữ liệu (≤ 5 MB) và backup hệ thống (Android data_extraction_rules / iCloud). Không mạng, không tài khoản.</t>
         </is>
       </c>
       <c r="E17" s="17" t="inlineStr">
@@ -1450,7 +1454,7 @@
       </c>
       <c r="G17" s="18" t="inlineStr">
         <is>
-          <t>Có importJson() nhưng chưa có UI (T-13).</t>
+          <t>Import + backup (T-13), test migration có fixture v1/v2 (T-35).</t>
         </is>
       </c>
     </row>
@@ -1472,7 +1476,7 @@
       </c>
       <c r="D18" s="18" t="inlineStr">
         <is>
-          <t>~130 chuỗi UI qua interface Strings (thiếu bản dịch → không compile), nội dung LocalizedText, DateFormat tự viết.</t>
+          <t>Toàn bộ chuỗi UI qua interface Strings (thiếu bản dịch → không compile), kể cả nhãn trợ năng; nội dung LocalizedText, DateFormat tự viết.</t>
         </is>
       </c>
       <c r="E18" s="17" t="inlineStr">
@@ -1485,7 +1489,7 @@
           <t>Hoàn thành</t>
         </is>
       </c>
-      <c r="G18" s="18" t="inlineStr"/>
+      <c r="G18" s="18" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="17" t="inlineStr">
@@ -1505,7 +1509,7 @@
       </c>
       <c r="D19" s="18" t="inlineStr">
         <is>
-          <t>120 thử thách (20/lĩnh vực × 6 lĩnh vực), 12 quote, bộ câu nhắc xoay vòng.</t>
+          <t>216 thử thách (36/lĩnh vực, mỗi lĩnh vực 12 Dễ / 12 Vừa / 12 Khó), 60 quote, bộ câu nhắc xoay vòng.</t>
         </is>
       </c>
       <c r="E19" s="17" t="inlineStr">
@@ -1520,7 +1524,7 @@
       </c>
       <c r="G19" s="18" t="inlineStr">
         <is>
-          <t>Spec nhắm ~240 thử thách cho beta.</t>
+          <t>Mở rộng ở T-26A/B. Còn: người dùng duyệt docs/content-review-challenges.md và thêm 96 id mới vào PublishedContent.kt trước khi phát hành.</t>
         </is>
       </c>
     </row>
@@ -1542,7 +1546,7 @@
       </c>
       <c r="D20" s="18" t="inlineStr">
         <is>
-          <t>67 test trong sharedLogic/commonTest chạy trên JVM và Kotlin/Native: streak, selector, stats, repository, kiểm tra toàn vẹn nội dung.</t>
+          <t>274 test sharedLogic/commonTest (JVM + Kotlin/Native): logic, migration, nội dung, tương phản màu, câu đọc trợ năng. UI test: Android 6 Compose test trên emulator, iOS 5 XCUITest (smoke, đổi ngày, 1 hoàn thành/ngày).</t>
         </is>
       </c>
       <c r="E20" s="17" t="inlineStr">
@@ -1552,12 +1556,12 @@
       </c>
       <c r="F20" s="17" t="inlineStr">
         <is>
-          <t>Một phần</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
       <c r="G20" s="18" t="inlineStr">
         <is>
-          <t>Chưa có UI test / instrumentation test cho Android &amp; iOS.</t>
+          <t>UI test thêm ở T-24. Luồng ngoài smoke vẫn QA tay.</t>
         </is>
       </c>
     </row>
@@ -1579,7 +1583,7 @@
       </c>
       <c r="D21" s="18" t="inlineStr">
         <is>
-          <t>Android: R8 + shrink resources, proguard cho serialization &amp; receivers, signing từ keystore.properties. iOS: iPhone-only, portrait, PrivacyInfo.xcprivacy, ITSAppUsesNonExemptEncryption=false, launch screen tối. Icon render từ 1 nguồn (tools/IconRenderer.swift). Có sẵn privacy policy HTML &amp; store listing song ngữ.</t>
+          <t>Android: R8 + shrink resources, proguard, signing từ keystore.properties, version từ iosApp/Configuration/Version.xcconfig (dùng chung). iOS: iPhone-only, portrait, deployment target 17.0, PrivacyInfo.xcprivacy, scheme dùng chung có UI test. Có privacy policy, store listing song ngữ, docs/release-process.md.</t>
         </is>
       </c>
       <c r="E21" s="17" t="inlineStr">
@@ -1594,7 +1598,7 @@
       </c>
       <c r="G21" s="18" t="inlineStr">
         <is>
-          <t>Còn placeholder: TEAM_ID, keystore, tên/ email nhà phát triển, link thương hiệu.</t>
+          <t>Version một nguồn + script bump (T-28), iOS 17 (T-18), giám sát crash không SDK (T-22). Còn placeholder: TEAM_ID, keystore, tên/email nhà phát triển, link thương hiệu (T-10, T-11, T-14…T-17).</t>
         </is>
       </c>
     </row>
@@ -2251,11 +2255,15 @@
       </c>
       <c r="J11" s="20" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Đang làm</t>
         </is>
       </c>
       <c r="K11" s="21" t="inlineStr"/>
-      <c r="L11" s="21" t="inlineStr"/>
+      <c r="L11" s="21" t="inlineStr">
+        <is>
+          <t>Code xong 25/10/2026: share card + caption dùng lil-dua.github.io/projects/oddly (Brand.WEBSITE_URL), bỏ handle @1percenthuman, giữ hashtag. Landing đã đăng (HTTP 200); bản thiết kế mới ở docs/landing/index.html cần đăng lại. Review APPROVE. Còn: QA thẻ share 9:16/1:1. Xem docs/plans/T-10_T-12.md.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="17" t="inlineStr">
@@ -2303,11 +2311,15 @@
       </c>
       <c r="J12" s="20" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Xong</t>
         </is>
       </c>
       <c r="K12" s="21" t="inlineStr"/>
-      <c r="L12" s="21" t="inlineStr"/>
+      <c r="L12" s="21" t="inlineStr">
+        <is>
+          <t>Xong 25/10/2026: điền nhà phát triển Lil Dua + email huuthom.it@gmail.com, host tại https://lil-dua.github.io/projects/oddly/privacy/privacy-policy.html (bản 19/10/2026, có backup/import/chẩn đoán). Nguồn: docs/privacy-policy.html — sửa xong phải đăng lại. Còn: dán URL vào Play Console / App Store Connect (T-16, T-17).</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="17" t="inlineStr">
@@ -2361,7 +2373,7 @@
       <c r="K13" s="21" t="inlineStr"/>
       <c r="L13" s="21" t="inlineStr">
         <is>
-          <t>Một phần 19/10/2026: version trong settingsFooter/aboutBody lấy từ build (BuildConfig.VERSION_NAME / CFBundleShortVersionString). Còn row Chính sách quyền riêng tư / Liên hệ / Đánh giá — chờ URL, email, link store (T-10/T-11).</t>
+          <t>Code xong 25/10/2026: mục "Hỗ trợ &amp; pháp lý" — Đánh giá (Android Play; iOS ẩn tới khi có APP_STORE_ID ở T-17), Liên hệ &amp; góp ý (email hiện dạng chữ), Chính sách quyền riêng tư, Giới thiệu (version từ build). Fallback sao chép địa chỉ khi không mở được. Review APPROVE. Còn: QA tay TalkBack/VoiceOver, điền APP_STORE_ID. Xem docs/plans/T-10_T-12.md.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Share card, remove shareUI, clear backlog
</commit_message>
<xml_diff>
--- a/docs/release-todo.xlsx
+++ b/docs/release-todo.xlsx
@@ -575,7 +575,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Phân tích mã nguồn ban đầu tại commit 8c842bf (18/10/2026); cập nhật tiến độ tại commit 73f905a, ngày 25/10/2026. Android (Compose) + iOS (SwiftUI) + sharedLogic (KMP).</t>
+          <t>Phân tích mã nguồn ban đầu tại commit 8c842bf (18/10/2026); cập nhật tiến độ tại commit a675129 + đợt T-30/T-31, ngày 25/10/2026. Android (Compose) + iOS (SwiftUI) + sharedLogic (KMP).</t>
         </is>
       </c>
     </row>
@@ -758,7 +758,7 @@
     <row r="15" ht="30" customHeight="1">
       <c r="A15" s="16" t="inlineStr">
         <is>
-          <t>• Kiến trúc tốt: logic dùng chung KMP, UI native, offline hoàn toàn, song ngữ. Có 274 unit test shared + UI test smoke (6 Android, 5 iOS), hỗ trợ TalkBack/VoiceOver, cỡ chữ lớn, màu chữ đạt WCAG AA.</t>
+          <t>• Kiến trúc tốt: logic dùng chung KMP, UI native, offline hoàn toàn, song ngữ. Có 303 unit test shared + UI test smoke (9 Android, 6 iOS), hỗ trợ TalkBack/VoiceOver, cỡ chữ lớn, màu chữ đạt WCAG AA.</t>
         </is>
       </c>
     </row>
@@ -772,7 +772,7 @@
     <row r="17" ht="30" customHeight="1">
       <c r="A17" s="16" t="inlineStr">
         <is>
-          <t>• Việc chặn phát hành còn lại cần người làm: thủ tục store (T-10, T-11, T-14…T-17, T-19…T-21), duyệt nội dung + xác minh nguồn quote (T-26, T-27), duyệt bảng màu neon theme Sáng (T-23C), QA tay thiết bị thật.</t>
+          <t>• Việc chặn phát hành còn lại cần người làm: thủ tục store (T-14…T-17, T-19…T-21), QA thẻ share (T-10), duyệt nội dung + xác minh nguồn quote (T-26, T-27), duyệt bảng màu neon theme Sáng (T-23C), QA tay thiết bị thật; đăng lại privacy policy (bản EN sửa "Erase").</t>
         </is>
       </c>
     </row>
@@ -2261,7 +2261,7 @@
       <c r="K11" s="21" t="inlineStr"/>
       <c r="L11" s="21" t="inlineStr">
         <is>
-          <t>Code xong 25/10/2026: share card + caption dùng lil-dua.github.io/projects/oddly (Brand.WEBSITE_URL), bỏ handle @1percenthuman, giữ hashtag. Landing đã đăng (HTTP 200); bản thiết kế mới ở docs/landing/index.html cần đăng lại. Review APPROVE. Còn: QA thẻ share 9:16/1:1. Xem docs/plans/T-10_T-12.md.</t>
+          <t>Code xong 25/10/2026: share card + caption dùng lil-dua.github.io/projects/oddly (Brand.WEBSITE_URL), bỏ handle @1percenthuman, giữ hashtag. Landing đã đăng (HTTP 200); bản thiết kế mới (docs/landing/index.html) đã đăng lại 25/10/2026. Review APPROVE. Còn: QA thẻ share 9:16/1:1. Xem docs/plans/T-10_T-12.md.</t>
         </is>
       </c>
     </row>
@@ -3335,11 +3335,19 @@
       </c>
       <c r="J31" s="20" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
-        </is>
-      </c>
-      <c r="K31" s="21" t="inlineStr"/>
-      <c r="L31" s="21" t="inlineStr"/>
+          <t>Xong</t>
+        </is>
+      </c>
+      <c r="K31" s="21" t="inlineStr">
+        <is>
+          <t>Claude (team-run)</t>
+        </is>
+      </c>
+      <c r="L31" s="21" t="inlineStr">
+        <is>
+          <t>Xong 25/10/2026: xoá sharedUI/ (3 file), gỡ alias catalog không dùng (core-ktx, espresso, testJunit), viết lại README, sửa comment ReminderScheduler/ReminderStore. bundleRelease OK. Review APPROVE (1 vòng sửa của cả đợt). Xem docs/plans/T-30_T-31_backlog.md.</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="17" t="inlineStr">
@@ -3387,11 +3395,19 @@
       </c>
       <c r="J32" s="20" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
-        </is>
-      </c>
-      <c r="K32" s="21" t="inlineStr"/>
-      <c r="L32" s="21" t="inlineStr"/>
+          <t>Đang làm</t>
+        </is>
+      </c>
+      <c r="K32" s="21" t="inlineStr">
+        <is>
+          <t>Claude (team-run)</t>
+        </is>
+      </c>
+      <c r="L32" s="21" t="inlineStr">
+        <is>
+          <t>Code xong 25/10/2026: ChallengeSeed.byId tra Map, selector O(n+m), swapsLeft overload không dựng PersistedState, StatsCalculator tính distribution 1 lần; Android derivedStateOf + completions List bất biến (sửa luôn CalendarScreen không tính lại), iOS stored property tính lại trong didSet. Cùng đợt dọn 10 mục backlog (câu mặt trời life_sunrise/life_watch_something_end, caption S08, S14 giữ chip lọc khi Share→Back, copy nhắc trung tính, privacy EN "Erase" — cần đăng lại site). 303 test shared, UI test Android 9/9, iOS 6/6. Review APPROVE (1 vòng sửa). Còn: QA tay (đổi range Statistics, qua nửa đêm, xoá/nhập backup, bản R8). Xem docs/plans/T-30_T-31_backlog.md.</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="17" t="inlineStr">

</xml_diff>

<commit_message>
Screen shot + CI github actions
</commit_message>
<xml_diff>
--- a/docs/release-todo.xlsx
+++ b/docs/release-todo.xlsx
@@ -575,7 +575,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Phân tích mã nguồn ban đầu tại commit 8c842bf (18/10/2026); cập nhật tiến độ tại commit a675129 + đợt T-30/T-31, ngày 25/10/2026. Android (Compose) + iOS (SwiftUI) + sharedLogic (KMP).</t>
+          <t>Phân tích mã nguồn ban đầu tại commit 8c842bf (18/10/2026); cập nhật tiến độ sau đợt T-19 + T-25, ngày 25/10/2026. Android (Compose) + iOS (SwiftUI) + sharedLogic (KMP).</t>
         </is>
       </c>
     </row>
@@ -758,7 +758,7 @@
     <row r="15" ht="30" customHeight="1">
       <c r="A15" s="16" t="inlineStr">
         <is>
-          <t>• Kiến trúc tốt: logic dùng chung KMP, UI native, offline hoàn toàn, song ngữ. Có 303 unit test shared + UI test smoke (9 Android, 6 iOS), hỗ trợ TalkBack/VoiceOver, cỡ chữ lớn, màu chữ đạt WCAG AA.</t>
+          <t>• Kiến trúc tốt: logic dùng chung KMP, UI native, offline hoàn toàn, song ngữ. Có 311 unit test shared + UI test smoke (9 Android, 6 iOS), CI GitHub Actions, script tự chụp ảnh store, hỗ trợ TalkBack/VoiceOver, cỡ chữ lớn, màu chữ đạt WCAG AA.</t>
         </is>
       </c>
     </row>
@@ -772,7 +772,7 @@
     <row r="17" ht="30" customHeight="1">
       <c r="A17" s="16" t="inlineStr">
         <is>
-          <t>• Việc chặn phát hành còn lại cần người làm: thủ tục store (T-14…T-17, T-19…T-21), QA thẻ share (T-10), duyệt nội dung + xác minh nguồn quote (T-26, T-27), duyệt bảng màu neon theme Sáng (T-23C), QA tay thiết bị thật; đăng lại privacy policy (bản EN sửa "Erase").</t>
+          <t>• Việc chặn phát hành còn lại cần người làm: thủ tục store (T-14…T-17, T-20, T-21), duyệt + tải ảnh store (T-19), QA thẻ share (T-10), duyệt nội dung + xác minh nguồn quote (T-26, T-27), duyệt bảng màu neon theme Sáng (T-23C), QA tay thiết bị thật; đăng lại privacy policy (bản EN sửa "Erase").</t>
         </is>
       </c>
     </row>
@@ -2739,11 +2739,19 @@
       </c>
       <c r="J20" s="20" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
-        </is>
-      </c>
-      <c r="K20" s="21" t="inlineStr"/>
-      <c r="L20" s="21" t="inlineStr"/>
+          <t>Đang làm</t>
+        </is>
+      </c>
+      <c r="K20" s="21" t="inlineStr">
+        <is>
+          <t>Claude (team-run)</t>
+        </is>
+      </c>
+      <c r="L20" s="21" t="inlineStr">
+        <is>
+          <t>Code xong 25/10/2026: tools/store-shots.sh sinh toàn bộ ảnh vào build/store-assets/ (~5 phút): Play 6 ảnh 1080×1920 vi/en + feature graphic 1024×500 vi/en + icon 512; App Store 6 ảnh 1320×2868 (iPhone 17 Pro Max) vi/en; có khung + caption theo store-listing §4, không alpha. Dữ liệu demo StoreShotScenario (chỉ test/DEBUG). Sửa kèm bug iOS: scrim che tiêu đề/nút đóng sheet chia sẻ. Review APPROVE (2 vòng sửa). Còn: duyệt caption + bộ ảnh, chọn 05-share Android 9:16 hay 1:1, tải lên store. Xem docs/plans/T-19.md.</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="17" t="inlineStr">
@@ -3059,11 +3067,19 @@
       </c>
       <c r="J26" s="20" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
-        </is>
-      </c>
-      <c r="K26" s="21" t="inlineStr"/>
-      <c r="L26" s="21" t="inlineStr"/>
+          <t>Đang làm</t>
+        </is>
+      </c>
+      <c r="K26" s="21" t="inlineStr">
+        <is>
+          <t>Claude (team-run)</t>
+        </is>
+      </c>
+      <c r="L26" s="21" t="inlineStr">
+        <is>
+          <t>Code xong 25/10/2026: .github/workflows/ci.yml (push/PR; job android: host test + lintDebug + bundleRelease không ký + compile androidTest; job ios macos-26: iosSimulatorArm64Test + xcodebuild build-for-testing) và ui-tests.yml (chạy tay). Lint baseline 40 issue cũ. actionlint 0 lỗi, lệnh chạy cục bộ xanh. Review APPROVE. Còn: push và xác nhận run đầu xanh trên GitHub (runner macos-26, Temurin 25) → chuyển Xong. Xem docs/plans/T-25.md.</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="17" t="inlineStr">

</xml_diff>